<commit_message>
Correct the Q8 reduction potential and rerun the benchmark
The reduction potential of Q8 was given against Fc+/Fc. It is now
-1.92 V vs SCE, as converted in the source (Patra et al., Nat. Catal.
2021), which removes PC25-Q8 from the scored set (855 pairs, 379
quenching). The Stern-Volmer read of PC25 batch 1 is updated.

Datasets, benchmark and further-analysis results are regenerated.
</commit_message>
<xml_diff>
--- a/data/exp_dataset.xlsx
+++ b/data/exp_dataset.xlsx
@@ -42058,13 +42058,13 @@
         </is>
       </c>
       <c r="G1155" s="10" t="n">
-        <v>56055.8</v>
+        <v>65108.3</v>
       </c>
       <c r="H1155" s="10" t="n">
         <v>6438.81</v>
       </c>
       <c r="I1155" s="10" t="n">
-        <v>8705930000</v>
+        <v>10111900000</v>
       </c>
       <c r="K1155" s="10" t="n">
         <v>1</v>
@@ -42094,13 +42094,13 @@
         </is>
       </c>
       <c r="G1156" s="10" t="n">
-        <v>49490.1</v>
+        <v>48151.8</v>
       </c>
       <c r="H1156" s="10" t="n">
         <v>6438.81</v>
       </c>
       <c r="I1156" s="10" t="n">
-        <v>7686220000</v>
+        <v>7478370000</v>
       </c>
       <c r="K1156" s="10" t="n">
         <v>1</v>
@@ -42130,13 +42130,13 @@
         </is>
       </c>
       <c r="G1157" s="10" t="n">
-        <v>61343.1</v>
+        <v>70862.5</v>
       </c>
       <c r="H1157" s="10" t="n">
         <v>6438.81</v>
       </c>
       <c r="I1157" s="10" t="n">
-        <v>9527090000</v>
+        <v>11005500000</v>
       </c>
       <c r="K1157" s="10" t="n">
         <v>1</v>
@@ -42166,13 +42166,13 @@
         </is>
       </c>
       <c r="G1158" s="10" t="n">
-        <v>37528.6</v>
+        <v>35177.8</v>
       </c>
       <c r="H1158" s="10" t="n">
         <v>6438.81</v>
       </c>
       <c r="I1158" s="10" t="n">
-        <v>5828500000</v>
+        <v>5463400000</v>
       </c>
       <c r="K1158" s="10" t="n">
         <v>1</v>
@@ -42202,13 +42202,13 @@
         </is>
       </c>
       <c r="G1159" s="10" t="n">
-        <v>59030.8</v>
+        <v>76748.2</v>
       </c>
       <c r="H1159" s="10" t="n">
         <v>6438.81</v>
       </c>
       <c r="I1159" s="10" t="n">
-        <v>9167970000</v>
+        <v>11919600000</v>
       </c>
       <c r="K1159" s="10" t="n">
         <v>1</v>
@@ -42238,13 +42238,13 @@
         </is>
       </c>
       <c r="G1160" s="10" t="n">
-        <v>54996.6</v>
+        <v>68358.8</v>
       </c>
       <c r="H1160" s="10" t="n">
         <v>6438.81</v>
       </c>
       <c r="I1160" s="10" t="n">
-        <v>8541420000</v>
+        <v>10616700000</v>
       </c>
       <c r="K1160" s="10" t="n">
         <v>1</v>
@@ -42274,13 +42274,13 @@
         </is>
       </c>
       <c r="G1161" s="10" t="n">
-        <v>54541.8</v>
+        <v>58402.4</v>
       </c>
       <c r="H1161" s="10" t="n">
         <v>6438.81</v>
       </c>
       <c r="I1161" s="10" t="n">
-        <v>8470790000</v>
+        <v>9070370000</v>
       </c>
       <c r="K1161" s="10" t="n">
         <v>1</v>
@@ -42310,13 +42310,13 @@
         </is>
       </c>
       <c r="G1162" s="10" t="n">
-        <v>18928.3</v>
+        <v>24189.7</v>
       </c>
       <c r="H1162" s="10" t="n">
         <v>6438.81</v>
       </c>
       <c r="I1162" s="10" t="n">
-        <v>2939720000</v>
+        <v>3756860000</v>
       </c>
       <c r="K1162" s="10" t="n">
         <v>1</v>
@@ -42346,13 +42346,13 @@
         </is>
       </c>
       <c r="G1163" s="10" t="n">
-        <v>44379.6</v>
+        <v>41263.1</v>
       </c>
       <c r="H1163" s="10" t="n">
         <v>6438.81</v>
       </c>
       <c r="I1163" s="10" t="n">
-        <v>6892520000</v>
+        <v>6408500000</v>
       </c>
       <c r="K1163" s="10" t="n">
         <v>1</v>
@@ -42382,13 +42382,13 @@
         </is>
       </c>
       <c r="G1164" s="10" t="n">
-        <v>35751.4</v>
+        <v>29516.4</v>
       </c>
       <c r="H1164" s="10" t="n">
         <v>6438.81</v>
       </c>
       <c r="I1164" s="10" t="n">
-        <v>5552490000</v>
+        <v>4584140000</v>
       </c>
       <c r="K1164" s="10" t="n">
         <v>1</v>
@@ -42418,13 +42418,13 @@
         </is>
       </c>
       <c r="G1165" s="10" t="n">
-        <v>1254.71</v>
+        <v>935.962</v>
       </c>
       <c r="H1165" s="10" t="n">
         <v>6438.81</v>
       </c>
       <c r="I1165" s="10" t="n">
-        <v>194867000</v>
+        <v>145363000</v>
       </c>
       <c r="K1165" s="10" t="n">
         <v>1</v>
@@ -42454,13 +42454,13 @@
         </is>
       </c>
       <c r="G1166" s="10" t="n">
-        <v>44061.9</v>
+        <v>42581.7</v>
       </c>
       <c r="H1166" s="10" t="n">
         <v>6438.81</v>
       </c>
       <c r="I1166" s="10" t="n">
-        <v>6843170000</v>
+        <v>6613290000</v>
       </c>
       <c r="K1166" s="10" t="n">
         <v>1</v>
@@ -42490,13 +42490,13 @@
         </is>
       </c>
       <c r="G1167" s="10" t="n">
-        <v>70579.7</v>
+        <v>81112.10000000001</v>
       </c>
       <c r="H1167" s="10" t="n">
         <v>6438.81</v>
       </c>
       <c r="I1167" s="10" t="n">
-        <v>10961600000</v>
+        <v>12597400000</v>
       </c>
       <c r="K1167" s="10" t="n">
         <v>1</v>
@@ -42526,13 +42526,13 @@
         </is>
       </c>
       <c r="G1168" s="10" t="n">
-        <v>8893.469999999999</v>
+        <v>10148.9</v>
       </c>
       <c r="H1168" s="10" t="n">
         <v>6438.81</v>
       </c>
       <c r="I1168" s="10" t="n">
-        <v>1381230000</v>
+        <v>1576210000</v>
       </c>
       <c r="K1168" s="10" t="n">
         <v>1</v>
@@ -42562,13 +42562,13 @@
         </is>
       </c>
       <c r="G1169" s="10" t="n">
-        <v>36886.2</v>
+        <v>46385.5</v>
       </c>
       <c r="H1169" s="10" t="n">
         <v>6438.81</v>
       </c>
       <c r="I1169" s="10" t="n">
-        <v>5728730000</v>
+        <v>7204050000</v>
       </c>
       <c r="K1169" s="10" t="n">
         <v>1</v>
@@ -42598,13 +42598,13 @@
         </is>
       </c>
       <c r="G1170" s="10" t="n">
-        <v>25029.4</v>
+        <v>37929.1</v>
       </c>
       <c r="H1170" s="10" t="n">
         <v>6438.81</v>
       </c>
       <c r="I1170" s="10" t="n">
-        <v>3887270000</v>
+        <v>5890700000</v>
       </c>
       <c r="K1170" s="10" t="n">
         <v>1</v>

</xml_diff>